<commit_message>
Use Excel-only batch and output templates
</commit_message>
<xml_diff>
--- a/data/templates/batch_input.xlsx
+++ b/data/templates/batch_input.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="R9e61144b41834fd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch_Input" sheetId="2" r:id="Rb06f0fbff24c4f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="Ra43ba63110d74cbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch_Input" sheetId="2" r:id="R007553869e314335"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -417,7 +417,7 @@
         <x:v>One row means</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>One new location to be processed by the feature pipeline and prediction API.</x:v>
+        <x:v>One new location to be processed by the feature pipeline and prediction model.</x:v>
       </x:c>
       <x:c r="C5" s="21"/>
       <x:c r="D5" s="21"/>
@@ -447,7 +447,7 @@
         <x:v>How to use</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>Enter or paste locations into Batch_Input without changing the headers. Add rows as needed, then submit the sheet through the agreed pipeline/API process.</x:v>
+        <x:v>Enter or paste locations into Batch_Input without changing the headers. Add rows as needed, then submit the workbook through the agreed pipeline process.</x:v>
       </x:c>
       <x:c r="C8" s="21"/>
       <x:c r="D8" s="21"/>
@@ -457,7 +457,7 @@
         <x:v>What happens next</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>The pipeline retrieves the deployed feature set, matches the road segment, runs the model and writes prediction_output.xlsx/CSV.</x:v>
+        <x:v>The pipeline retrieves the deployed feature set, matches the road segment, runs the model and writes results to prediction_output.xlsx.</x:v>
       </x:c>
       <x:c r="C9" s="21"/>
       <x:c r="D9" s="21"/>
@@ -467,7 +467,7 @@
         <x:v>Git / sharing</x:v>
       </x:c>
       <x:c r="B10" s="21" t="str">
-        <x:v>The blank template can be stored in Git. A filled workbook should follow the project’s approved data-sharing rules.</x:v>
+        <x:v>The blank Excel template can be stored in Git. A filled workbook should follow the project’s approved data-sharing rules.</x:v>
       </x:c>
       <x:c r="C10" s="21"/>
       <x:c r="D10" s="21"/>
@@ -1063,7 +1063,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2acb4e368f304aef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb41486c5ff54f25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>